<commit_message>
feat(lead_magnet): standardize naming to 2026外贸出厂底价表与智能核价模板_Kelvin旗舰版
</commit_message>
<xml_diff>
--- a/lead_magnets/2026_外贸出厂核算控制台与批量算价神表_Kelvin旗舰版_新对齐.xlsx
+++ b/lead_magnets/2026_外贸出厂核算控制台与批量算价神表_Kelvin旗舰版_新对齐.xlsx
@@ -1,15 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\xhs_operator\lead_magnets\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <bookViews>
+    <workbookView windowWidth="22188" windowHeight="9060"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="📌 使用指南与提效神器" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="⚙️ 全局核算参数 (Config)" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="📦 商品出厂底价库 (Products)" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="📄 对外纯净批量报价单 (脱敏单)" state="visible" r:id="rId7"/>
+    <sheet name="📌 使用指南与提效神器" sheetId="1" r:id="rId1"/>
+    <sheet name="⚙️ 全局核算参数 (Config)" sheetId="2" r:id="rId2"/>
+    <sheet name="📦 商品出厂底价库 (Products)" sheetId="3" r:id="rId3"/>
+    <sheet name="📄 对外纯净批量报价单 (脱敏单)" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -505,136 +526,310 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="8">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="¥#,##0.00"/>
-    <numFmt numFmtId="167" formatCode="+0.0%;-0.0%;0.0%"/>
-    <numFmt numFmtId="168" formatCode="0.0&quot; CBM&quot;"/>
-    <numFmt numFmtId="169" formatCode="#,##0&quot; KG&quot;"/>
-    <numFmt numFmtId="170" formatCode="0.000"/>
-    <numFmt numFmtId="171" formatCode="$#,##0.00"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="12">
+    <numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="42" formatCode="_(&quot;HK$&quot;* #,##0_);_(&quot;HK$&quot;* \(#,##0\);_(&quot;HK$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_(&quot;HK$&quot;* #,##0.00_);_(&quot;HK$&quot;* \(#,##0.00\);_(&quot;HK$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="177" formatCode="\$#,##0.00"/>
+    <numFmt numFmtId="178" formatCode="\¥#,##0.00"/>
+    <numFmt numFmtId="179" formatCode="0.000"/>
+    <numFmt numFmtId="180" formatCode="0.0"/>
+    <numFmt numFmtId="181" formatCode="0.0%"/>
+    <numFmt numFmtId="182" formatCode="\+0.0%;\-0.0%;0.0%"/>
+    <numFmt numFmtId="183" formatCode="0.0&quot; CBM&quot;"/>
+    <numFmt numFmtId="184" formatCode="#,##0&quot; KG&quot;"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
-    <font>
+  <fonts count="40">
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
-      <family val="2"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9.5"/>
+      <color rgb="FF1E293B"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="9.5"/>
+      <color rgb="FF1E293B"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1E3A8A"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10.5"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Microsoft YaHei"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="9.5"/>
+      <color rgb="FF1E293B"/>
+      <name val="Microsoft YaHei"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9.5"/>
+      <color rgb="FF1E293B"/>
+      <name val="Microsoft YaHei"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9.5"/>
+      <color rgb="FF1E3A8A"/>
+      <name val="Microsoft YaHei"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Microsoft YaHei"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="9.5"/>
+      <color rgb="FF475569"/>
+      <name val="Microsoft YaHei"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
-      <name val="Calibri"/>
+      <color rgb="FF1E3A8A"/>
+      <name val="Microsoft YaHei"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Microsoft YaHei"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1E293B"/>
+      <name val="Microsoft YaHei"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1E293B"/>
+      <name val="Microsoft YaHei"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFB91C1C"/>
+      <name val="Microsoft YaHei"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFB91C1C"/>
+      <name val="Microsoft YaHei"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9.5"/>
+      <color rgb="FF475569"/>
+      <name val="Microsoft YaHei"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1E3A8A"/>
+      <name val="Microsoft YaHei"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="13"/>
-      <name val="Microsoft YaHei"/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="FF475569"/>
-      <sz val="9.5"/>
-      <name val="Microsoft YaHei"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF1E3A8A"/>
-      <sz val="10"/>
-      <name val="Microsoft YaHei"/>
-    </font>
-    <font>
-      <color rgb="FF1E293B"/>
-      <sz val="9.5"/>
-      <name val="Microsoft YaHei"/>
-    </font>
-    <font>
-      <color rgb="FF475569"/>
-      <sz val="9.5"/>
-      <name val="Microsoft YaHei"/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF1E3A8A"/>
       <sz val="11"/>
-      <name val="Microsoft YaHei"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
-      <name val="Microsoft YaHei"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF1E293B"/>
-      <sz val="10"/>
-      <name val="Microsoft YaHei"/>
-    </font>
-    <font>
-      <color rgb="FF1E293B"/>
-      <sz val="10"/>
-      <name val="Microsoft YaHei"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFB91C1C"/>
-      <sz val="10"/>
-      <name val="Microsoft YaHei"/>
-    </font>
-    <font>
-      <color rgb="FFB91C1C"/>
-      <sz val="10"/>
-      <name val="Microsoft YaHei"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="10.5"/>
-      <name val="Microsoft YaHei"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF1E293B"/>
-      <sz val="9.5"/>
-      <name val="Microsoft YaHei"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF1E3A8A"/>
-      <sz val="9.5"/>
-      <name val="Microsoft YaHei"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="13"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="FF1E293B"/>
-      <sz val="9.5"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <color rgb="FF1E293B"/>
-      <sz val="9.5"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF1E3A8A"/>
-      <sz val="10"/>
-      <name val="Arial"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="40">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -644,40 +839,233 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1E3A8A"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF8FAFC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2563EB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD97706"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF3C7"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDBEAFE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF2563EB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD97706"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFEF3C7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -700,9 +1088,251 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="11" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="12" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -710,103 +1340,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="9" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="9" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -814,34 +1354,10 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="13" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="14" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -850,69 +1366,227 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="13" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="7" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="7" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="9" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="3" fontId="18" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="19" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="3" fontId="18" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="19" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="14" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="16" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="14" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="15" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="15" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="15" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="15" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="15" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="184" fontId="15" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="15" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="184" fontId="15" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  <cellStyles count="49">
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1234,77 +1908,77 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="B2:C10"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="85" customWidth="1"/>
+    <col min="2" max="2" width="42.8888888888889" customWidth="1"/>
+    <col min="3" max="3" width="100.666666666667" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" ht="38" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B2" s="1" t="s">
+    <row r="2" ht="38" customHeight="1" spans="2:3">
+      <c r="B2" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1"/>
-    </row>
-    <row r="3" ht="24" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B3" s="2" t="s">
+      <c r="C2" s="34"/>
+    </row>
+    <row r="3" ht="24" customHeight="1" spans="2:3">
+      <c r="B3" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="2"/>
-    </row>
-    <row r="5" ht="36" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="3" t="s">
+      <c r="C3" s="62"/>
+    </row>
+    <row r="5" ht="36" customHeight="1" spans="2:3">
+      <c r="B5" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="64" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" ht="36" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B6" s="3" t="s">
+    <row r="6" ht="36" customHeight="1" spans="2:3">
+      <c r="B6" s="63" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="65" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B7" s="3" t="s">
+    <row r="7" ht="36" customHeight="1" spans="2:3">
+      <c r="B7" s="63" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="64" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" ht="36" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="3" t="s">
+    <row r="8" ht="36" customHeight="1" spans="2:3">
+      <c r="B8" s="63" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="65" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" ht="36" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B9" s="3" t="s">
+    <row r="9" ht="50" customHeight="1" spans="2:3">
+      <c r="B9" s="63" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="64" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" ht="36" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B10" s="3" t="s">
+    <row r="10" ht="36" customHeight="1" spans="2:3">
+      <c r="B10" s="63" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="65" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1314,14 +1988,16 @@
     <mergeCell ref="B3:C3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:E35"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
@@ -1330,457 +2006,457 @@
     <col min="5" max="5" width="54" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="38" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="38" customHeight="1" spans="1:5">
+      <c r="A1" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="2" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+    </row>
+    <row r="2" ht="24" customHeight="1" spans="1:5">
+      <c r="A2" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-    </row>
-    <row r="4" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+    </row>
+    <row r="4" ht="26" customHeight="1" spans="1:5">
+      <c r="A4" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-    </row>
-    <row r="5" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+      <c r="B4" s="36"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="36"/>
+    </row>
+    <row r="5" ht="24" customHeight="1" spans="1:5">
+      <c r="A5" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="37" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="37" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
+    <row r="6" ht="22" customHeight="1" spans="1:5">
+      <c r="A6" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="39">
         <v>7.2</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="D6" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="E6" s="41" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+    <row r="7" ht="22" customHeight="1" spans="1:5">
+      <c r="A7" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="14">
+      <c r="B7" s="43">
         <v>7.85</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="C7" s="44" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="16" t="s">
+      <c r="D7" s="45" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="16" t="s">
+      <c r="E7" s="45" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
+    <row r="8" ht="22" customHeight="1" spans="1:5">
+      <c r="A8" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="10">
+      <c r="B8" s="39">
         <v>9.1</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="40" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="D8" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="E8" s="41" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="13" t="s">
+    <row r="9" ht="22" customHeight="1" spans="1:5">
+      <c r="A9" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="14">
+      <c r="B9" s="43">
         <v>4.8</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="C9" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="45" t="s">
         <v>28</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="E9" s="45" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
+    <row r="10" ht="22" customHeight="1" spans="1:5">
+      <c r="A10" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="39">
         <v>5.3</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="12" t="s">
+      <c r="E10" s="41" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="12" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
+    <row r="12" ht="26" customHeight="1" spans="1:5">
+      <c r="A12" s="36" t="s">
         <v>39</v>
       </c>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-    </row>
-    <row r="13" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
+      <c r="B12" s="36"/>
+      <c r="C12" s="36"/>
+      <c r="D12" s="36"/>
+      <c r="E12" s="36"/>
+    </row>
+    <row r="13" ht="24" customHeight="1" spans="1:5">
+      <c r="A13" s="37" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="37" t="s">
         <v>42</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="37" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="17" t="s">
+    <row r="14" ht="22" customHeight="1" spans="1:5">
+      <c r="A14" s="46" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="18">
+      <c r="B14" s="47">
         <v>0.15</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="40" t="s">
         <v>46</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="D14" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="E14" s="12" t="s">
+      <c r="E14" s="41" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="19" t="s">
+    <row r="15" ht="22" customHeight="1" spans="1:5">
+      <c r="A15" s="48" t="s">
         <v>49</v>
       </c>
-      <c r="B15" s="20">
+      <c r="B15" s="49">
         <v>0.08</v>
       </c>
-      <c r="C15" s="21" t="s">
+      <c r="C15" s="50" t="s">
         <v>50</v>
       </c>
-      <c r="D15" s="22" t="s">
+      <c r="D15" s="51" t="s">
         <v>51</v>
       </c>
-      <c r="E15" s="22" t="s">
+      <c r="E15" s="51" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="17" t="s">
+    <row r="16" ht="22" customHeight="1" spans="1:5">
+      <c r="A16" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="B16" s="23">
+      <c r="B16" s="52">
         <v>2.5</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="40" t="s">
         <v>54</v>
       </c>
-      <c r="D16" s="12" t="s">
+      <c r="D16" s="41" t="s">
         <v>55</v>
       </c>
-      <c r="E16" s="12" t="s">
+      <c r="E16" s="41" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="24" t="s">
+    <row r="17" ht="22" customHeight="1" spans="1:5">
+      <c r="A17" s="53" t="s">
         <v>57</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B17" s="42" t="s">
         <v>58</v>
       </c>
-      <c r="C17" s="15" t="s">
+      <c r="C17" s="44" t="s">
         <v>59</v>
       </c>
-      <c r="D17" s="16" t="s">
+      <c r="D17" s="45" t="s">
         <v>60</v>
       </c>
-      <c r="E17" s="16" t="s">
+      <c r="E17" s="45" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="19" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
+    <row r="19" ht="26" customHeight="1" spans="1:5">
+      <c r="A19" s="36" t="s">
         <v>62</v>
       </c>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-    </row>
-    <row r="20" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="8" t="s">
+      <c r="B19" s="36"/>
+      <c r="C19" s="36"/>
+      <c r="D19" s="36"/>
+      <c r="E19" s="36"/>
+    </row>
+    <row r="20" ht="24" customHeight="1" spans="1:5">
+      <c r="A20" s="37" t="s">
         <v>63</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="37" t="s">
         <v>65</v>
       </c>
-      <c r="D20" s="8" t="s">
+      <c r="D20" s="37" t="s">
         <v>66</v>
       </c>
-      <c r="E20" s="8" t="s">
+      <c r="E20" s="37" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="21" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="9" t="s">
+    <row r="21" ht="22" customHeight="1" spans="1:5">
+      <c r="A21" s="38" t="s">
         <v>68</v>
       </c>
-      <c r="B21" s="12" t="s">
+      <c r="B21" s="41" t="s">
         <v>69</v>
       </c>
-      <c r="C21" s="25">
+      <c r="C21" s="54">
         <v>0</v>
       </c>
-      <c r="D21" s="25">
+      <c r="D21" s="54">
         <v>0</v>
       </c>
-      <c r="E21" s="12" t="s">
+      <c r="E21" s="41" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="22" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="13" t="s">
+    <row r="22" ht="22" customHeight="1" spans="1:5">
+      <c r="A22" s="42" t="s">
         <v>71</v>
       </c>
-      <c r="B22" s="16" t="s">
+      <c r="B22" s="45" t="s">
         <v>72</v>
       </c>
-      <c r="C22" s="26">
+      <c r="C22" s="55">
         <v>0.2</v>
       </c>
-      <c r="D22" s="26">
+      <c r="D22" s="55">
         <v>1500</v>
       </c>
-      <c r="E22" s="16" t="s">
+      <c r="E22" s="45" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="23" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="9" t="s">
+    <row r="23" ht="22" customHeight="1" spans="1:5">
+      <c r="A23" s="38" t="s">
         <v>74</v>
       </c>
-      <c r="B23" s="12" t="s">
+      <c r="B23" s="41" t="s">
         <v>75</v>
       </c>
-      <c r="C23" s="11" t="s">
+      <c r="C23" s="40" t="s">
         <v>76</v>
       </c>
-      <c r="D23" s="11" t="s">
+      <c r="D23" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="E23" s="12" t="s">
+      <c r="E23" s="41" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="25" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="7" t="s">
+    <row r="25" ht="26" customHeight="1" spans="1:5">
+      <c r="A25" s="36" t="s">
         <v>79</v>
       </c>
-      <c r="B25" s="7"/>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
-    </row>
-    <row r="26" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="8" t="s">
+      <c r="B25" s="36"/>
+      <c r="C25" s="36"/>
+      <c r="D25" s="36"/>
+      <c r="E25" s="36"/>
+    </row>
+    <row r="26" ht="24" customHeight="1" spans="1:5">
+      <c r="A26" s="37" t="s">
         <v>80</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="37" t="s">
         <v>81</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="37" t="s">
         <v>82</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="D26" s="37" t="s">
         <v>83</v>
       </c>
-      <c r="E26" s="8" t="s">
+      <c r="E26" s="37" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="27" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="17" t="s">
+    <row r="27" ht="22" customHeight="1" spans="1:5">
+      <c r="A27" s="46" t="s">
         <v>85</v>
       </c>
-      <c r="B27" s="27">
+      <c r="B27" s="56">
         <v>-0.02</v>
       </c>
-      <c r="C27" s="11" t="s">
+      <c r="C27" s="40" t="s">
         <v>86</v>
       </c>
-      <c r="D27" s="12" t="s">
+      <c r="D27" s="41" t="s">
         <v>87</v>
       </c>
-      <c r="E27" s="12" t="s">
+      <c r="E27" s="41" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="28" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="24" t="s">
+    <row r="28" ht="22" customHeight="1" spans="1:5">
+      <c r="A28" s="53" t="s">
         <v>89</v>
       </c>
-      <c r="B28" s="28">
+      <c r="B28" s="57">
         <v>0</v>
       </c>
-      <c r="C28" s="15" t="s">
+      <c r="C28" s="44" t="s">
         <v>86</v>
       </c>
-      <c r="D28" s="16" t="s">
+      <c r="D28" s="45" t="s">
         <v>90</v>
       </c>
-      <c r="E28" s="16" t="s">
+      <c r="E28" s="45" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="29" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="17" t="s">
+    <row r="29" ht="22" customHeight="1" spans="1:5">
+      <c r="A29" s="46" t="s">
         <v>92</v>
       </c>
-      <c r="B29" s="27">
+      <c r="B29" s="56">
         <v>0.015</v>
       </c>
-      <c r="C29" s="11" t="s">
+      <c r="C29" s="40" t="s">
         <v>93</v>
       </c>
-      <c r="D29" s="12" t="s">
+      <c r="D29" s="41" t="s">
         <v>94</v>
       </c>
-      <c r="E29" s="12" t="s">
+      <c r="E29" s="41" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="31" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="7" t="s">
+    <row r="31" ht="26" customHeight="1" spans="1:5">
+      <c r="A31" s="36" t="s">
         <v>96</v>
       </c>
-      <c r="B31" s="7"/>
-      <c r="C31" s="7"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
-    </row>
-    <row r="32" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="8" t="s">
+      <c r="B31" s="36"/>
+      <c r="C31" s="36"/>
+      <c r="D31" s="36"/>
+      <c r="E31" s="36"/>
+    </row>
+    <row r="32" ht="24" customHeight="1" spans="1:5">
+      <c r="A32" s="37" t="s">
         <v>97</v>
       </c>
-      <c r="B32" s="8" t="s">
+      <c r="B32" s="37" t="s">
         <v>98</v>
       </c>
-      <c r="C32" s="8" t="s">
+      <c r="C32" s="37" t="s">
         <v>99</v>
       </c>
-      <c r="D32" s="8" t="s">
+      <c r="D32" s="37" t="s">
         <v>100</v>
       </c>
-      <c r="E32" s="8" t="s">
+      <c r="E32" s="37" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="33" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="17" t="s">
+    <row r="33" ht="22" customHeight="1" spans="1:5">
+      <c r="A33" s="46" t="s">
         <v>102</v>
       </c>
-      <c r="B33" s="29">
+      <c r="B33" s="58">
         <v>28</v>
       </c>
-      <c r="C33" s="29">
+      <c r="C33" s="58">
         <v>33.2</v>
       </c>
-      <c r="D33" s="30">
+      <c r="D33" s="59">
         <v>21800</v>
       </c>
-      <c r="E33" s="12" t="s">
+      <c r="E33" s="41" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="34" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="24" t="s">
+    <row r="34" ht="22" customHeight="1" spans="1:5">
+      <c r="A34" s="53" t="s">
         <v>104</v>
       </c>
-      <c r="B34" s="31">
+      <c r="B34" s="60">
         <v>58</v>
       </c>
-      <c r="C34" s="31">
+      <c r="C34" s="60">
         <v>67.7</v>
       </c>
-      <c r="D34" s="32">
+      <c r="D34" s="61">
         <v>26000</v>
       </c>
-      <c r="E34" s="16" t="s">
+      <c r="E34" s="45" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="35" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="17" t="s">
+    <row r="35" ht="22" customHeight="1" spans="1:5">
+      <c r="A35" s="46" t="s">
         <v>106</v>
       </c>
-      <c r="B35" s="29">
+      <c r="B35" s="58">
         <v>68</v>
       </c>
-      <c r="C35" s="29">
+      <c r="C35" s="58">
         <v>76.3</v>
       </c>
-      <c r="D35" s="30">
+      <c r="D35" s="59">
         <v>26000</v>
       </c>
-      <c r="E35" s="12" t="s">
+      <c r="E35" s="41" t="s">
         <v>107</v>
       </c>
     </row>
@@ -1795,14 +2471,16 @@
     <mergeCell ref="A31:E31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:Q7"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="6"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="55" customWidth="1"/>
@@ -1820,379 +2498,417 @@
     <col min="17" max="17" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A1" s="33" t="s">
+    <row r="1" ht="32" customHeight="1" spans="1:17">
+      <c r="A1" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="C1" s="33" t="s">
+      <c r="C1" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="D1" s="33" t="s">
+      <c r="D1" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="E1" s="33" t="s">
+      <c r="E1" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="F1" s="33" t="s">
+      <c r="F1" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="G1" s="33" t="s">
+      <c r="G1" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="H1" s="33" t="s">
+      <c r="H1" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="I1" s="33" t="s">
+      <c r="I1" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="J1" s="33" t="s">
+      <c r="J1" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="K1" s="33" t="s">
+      <c r="K1" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="L1" s="34" t="s">
+      <c r="L1" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="M1" s="34" t="s">
+      <c r="M1" s="14" t="s">
         <v>120</v>
       </c>
-      <c r="N1" s="34" t="s">
+      <c r="N1" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="O1" s="34" t="s">
+      <c r="O1" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="P1" s="34" t="s">
+      <c r="P1" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="Q1" s="34" t="s">
+      <c r="Q1" s="14" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="2" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="35" t="s">
+    <row r="2" ht="24" customHeight="1" spans="1:17">
+      <c r="A2" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="16" t="s">
         <v>126</v>
       </c>
-      <c r="C2" s="36" t="s">
+      <c r="C2" s="16" t="s">
         <v>127</v>
       </c>
-      <c r="D2" s="37">
+      <c r="D2" s="17">
         <v>15.5</v>
       </c>
-      <c r="E2" s="38">
-        <v>500</v>
-      </c>
-      <c r="F2" s="38">
+      <c r="E2" s="18">
+        <v>600</v>
+      </c>
+      <c r="F2" s="18">
         <v>50</v>
       </c>
-      <c r="G2" s="39">
+      <c r="G2" s="19">
         <v>0.045</v>
       </c>
-      <c r="H2" s="40">
+      <c r="H2" s="20">
         <v>14.5</v>
       </c>
-      <c r="I2" s="41"/>
-      <c r="J2" s="35" t="s">
+      <c r="I2" s="21"/>
+      <c r="J2" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="K2" s="35" t="s">
+      <c r="K2" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="L2" s="42">
+      <c r="L2" s="22">
         <f>'⚙️ 全局核算参数 (Config)'!$C$22</f>
-      </c>
-      <c r="M2" s="43">
-        <f>IF(ISBLANK(I2), '⚙️ 全局核算参数 (Config)'!$B$14, I2)</f>
-      </c>
-      <c r="N2" s="44">
-        <f>ROUND(((D2 * (1 + M2) + L2) / '⚙️ 全局核算参数 (Config)'!$B$6), 2)</f>
-      </c>
-      <c r="O2" s="45">
-        <f>IF(AND(G2&gt;0, F2&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$33 / G2)) * F2, "-")</f>
-      </c>
-      <c r="P2" s="45">
-        <f>IF(AND(G2&gt;0, F2&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$35 / G2)) * F2, "-")</f>
-      </c>
-      <c r="Q2" s="46">
-        <f>IF(M2&lt;'⚙️ 全局核算参数 (Config)'!$B$15, "🚨 穿透红线", IF(M2&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
-      </c>
-    </row>
-    <row r="3" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" s="47" t="s">
+        <v>0.2</v>
+      </c>
+      <c r="M2" s="23">
+        <f>IF(ISBLANK(I2),'⚙️ 全局核算参数 (Config)'!$B$14,I2)</f>
+        <v>0.15</v>
+      </c>
+      <c r="N2" s="24">
+        <f>ROUND(((D2*(1+M2)+L2)/'⚙️ 全局核算参数 (Config)'!$B$6),2)</f>
+        <v>2.5</v>
+      </c>
+      <c r="O2" s="25">
+        <f>IF(AND(G2&gt;0,F2&gt;0),INT(('⚙️ 全局核算参数 (Config)'!$B$33/G2))*F2,"-")</f>
+        <v>31100</v>
+      </c>
+      <c r="P2" s="25">
+        <f>IF(AND(G2&gt;0,F2&gt;0),INT(('⚙️ 全局核算参数 (Config)'!$B$35/G2))*F2,"-")</f>
+        <v>75550</v>
+      </c>
+      <c r="Q2" s="26" t="str">
+        <f>IF(M2&lt;'⚙️ 全局核算参数 (Config)'!$B$15,"🚨 穿透红线",IF(M2&gt;=0.25,"💎 高毛利款","✅ 利润健康"))</f>
+        <v>✅ 利润健康</v>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1" spans="1:17">
+      <c r="A3" s="27" t="s">
         <v>130</v>
       </c>
-      <c r="B3" s="48" t="s">
+      <c r="B3" s="28" t="s">
         <v>131</v>
       </c>
-      <c r="C3" s="48" t="s">
+      <c r="C3" s="28" t="s">
         <v>132</v>
       </c>
-      <c r="D3" s="49">
+      <c r="D3" s="29">
         <v>0.85</v>
       </c>
-      <c r="E3" s="50">
+      <c r="E3" s="30">
         <v>5000</v>
       </c>
-      <c r="F3" s="50">
+      <c r="F3" s="30">
         <v>1000</v>
       </c>
-      <c r="G3" s="51">
+      <c r="G3" s="31">
         <v>0.02</v>
       </c>
-      <c r="H3" s="52">
+      <c r="H3" s="32">
         <v>18</v>
       </c>
-      <c r="I3" s="53">
+      <c r="I3" s="33">
         <v>0.18</v>
       </c>
-      <c r="J3" s="47" t="s">
+      <c r="J3" s="27" t="s">
         <v>133</v>
       </c>
-      <c r="K3" s="47" t="s">
+      <c r="K3" s="27" t="s">
         <v>134</v>
       </c>
-      <c r="L3" s="42">
+      <c r="L3" s="22">
         <f>'⚙️ 全局核算参数 (Config)'!$C$22</f>
-      </c>
-      <c r="M3" s="43">
-        <f>IF(ISBLANK(I3), '⚙️ 全局核算参数 (Config)'!$B$14, I3)</f>
-      </c>
-      <c r="N3" s="44">
-        <f>ROUND(((D3 * (1 + M3) + L3) / '⚙️ 全局核算参数 (Config)'!$B$6), 2)</f>
-      </c>
-      <c r="O3" s="45">
-        <f>IF(AND(G3&gt;0, F3&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$33 / G3)) * F3, "-")</f>
-      </c>
-      <c r="P3" s="45">
-        <f>IF(AND(G3&gt;0, F3&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$35 / G3)) * F3, "-")</f>
-      </c>
-      <c r="Q3" s="46">
-        <f>IF(M3&lt;'⚙️ 全局核算参数 (Config)'!$B$15, "🚨 穿透红线", IF(M3&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
-      </c>
-    </row>
-    <row r="4" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4" s="35" t="s">
+        <v>0.2</v>
+      </c>
+      <c r="M3" s="23">
+        <f>IF(ISBLANK(I3),'⚙️ 全局核算参数 (Config)'!$B$14,I3)</f>
+        <v>0.18</v>
+      </c>
+      <c r="N3" s="24">
+        <f>ROUND(((D3*(1+M3)+L3)/'⚙️ 全局核算参数 (Config)'!$B$6),2)</f>
+        <v>0.17</v>
+      </c>
+      <c r="O3" s="25">
+        <f>IF(AND(G3&gt;0,F3&gt;0),INT(('⚙️ 全局核算参数 (Config)'!$B$33/G3))*F3,"-")</f>
+        <v>1400000</v>
+      </c>
+      <c r="P3" s="25">
+        <f>IF(AND(G3&gt;0,F3&gt;0),INT(('⚙️ 全局核算参数 (Config)'!$B$35/G3))*F3,"-")</f>
+        <v>3400000</v>
+      </c>
+      <c r="Q3" s="26" t="str">
+        <f>IF(M3&lt;'⚙️ 全局核算参数 (Config)'!$B$15,"🚨 穿透红线",IF(M3&gt;=0.25,"💎 高毛利款","✅ 利润健康"))</f>
+        <v>✅ 利润健康</v>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1" spans="1:17">
+      <c r="A4" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="16" t="s">
         <v>136</v>
       </c>
-      <c r="C4" s="36" t="s">
+      <c r="C4" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="D4" s="37">
+      <c r="D4" s="17">
         <v>185</v>
       </c>
-      <c r="E4" s="38">
+      <c r="E4" s="18">
         <v>50</v>
       </c>
-      <c r="F4" s="38">
+      <c r="F4" s="18">
         <v>1</v>
       </c>
-      <c r="G4" s="39">
+      <c r="G4" s="19">
         <v>0.16</v>
       </c>
-      <c r="H4" s="40">
+      <c r="H4" s="20">
         <v>16.2</v>
       </c>
-      <c r="I4" s="41">
+      <c r="I4" s="21">
         <v>0.25</v>
       </c>
-      <c r="J4" s="35" t="s">
+      <c r="J4" s="15" t="s">
         <v>138</v>
       </c>
-      <c r="K4" s="35" t="s">
+      <c r="K4" s="15" t="s">
         <v>139</v>
       </c>
-      <c r="L4" s="42">
+      <c r="L4" s="22">
         <f>'⚙️ 全局核算参数 (Config)'!$C$22</f>
-      </c>
-      <c r="M4" s="43">
-        <f>IF(ISBLANK(I4), '⚙️ 全局核算参数 (Config)'!$B$14, I4)</f>
-      </c>
-      <c r="N4" s="44">
-        <f>ROUND(((D4 * (1 + M4) + L4) / '⚙️ 全局核算参数 (Config)'!$B$6), 2)</f>
-      </c>
-      <c r="O4" s="45">
-        <f>IF(AND(G4&gt;0, F4&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$33 / G4)) * F4, "-")</f>
-      </c>
-      <c r="P4" s="45">
-        <f>IF(AND(G4&gt;0, F4&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$35 / G4)) * F4, "-")</f>
-      </c>
-      <c r="Q4" s="46">
-        <f>IF(M4&lt;'⚙️ 全局核算参数 (Config)'!$B$15, "🚨 穿透红线", IF(M4&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
-      </c>
-    </row>
-    <row r="5" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A5" s="47" t="s">
+        <v>0.2</v>
+      </c>
+      <c r="M4" s="23">
+        <f>IF(ISBLANK(I4),'⚙️ 全局核算参数 (Config)'!$B$14,I4)</f>
+        <v>0.25</v>
+      </c>
+      <c r="N4" s="24">
+        <f>ROUND(((D4*(1+M4)+L4)/'⚙️ 全局核算参数 (Config)'!$B$6),2)</f>
+        <v>32.15</v>
+      </c>
+      <c r="O4" s="25">
+        <f>IF(AND(G4&gt;0,F4&gt;0),INT(('⚙️ 全局核算参数 (Config)'!$B$33/G4))*F4,"-")</f>
+        <v>175</v>
+      </c>
+      <c r="P4" s="25">
+        <f>IF(AND(G4&gt;0,F4&gt;0),INT(('⚙️ 全局核算参数 (Config)'!$B$35/G4))*F4,"-")</f>
+        <v>425</v>
+      </c>
+      <c r="Q4" s="26" t="str">
+        <f>IF(M4&lt;'⚙️ 全局核算参数 (Config)'!$B$15,"🚨 穿透红线",IF(M4&gt;=0.25,"💎 高毛利款","✅ 利润健康"))</f>
+        <v>💎 高毛利款</v>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1" spans="1:17">
+      <c r="A5" s="27" t="s">
         <v>140</v>
       </c>
-      <c r="B5" s="48" t="s">
+      <c r="B5" s="28" t="s">
         <v>141</v>
       </c>
-      <c r="C5" s="48" t="s">
+      <c r="C5" s="28" t="s">
         <v>142</v>
       </c>
-      <c r="D5" s="49">
+      <c r="D5" s="29">
         <v>38</v>
       </c>
-      <c r="E5" s="50">
+      <c r="E5" s="30">
         <v>200</v>
       </c>
-      <c r="F5" s="50">
+      <c r="F5" s="30">
         <v>5</v>
       </c>
-      <c r="G5" s="51">
+      <c r="G5" s="31">
         <v>0.08</v>
       </c>
-      <c r="H5" s="52">
+      <c r="H5" s="32">
         <v>11</v>
       </c>
-      <c r="I5" s="53"/>
-      <c r="J5" s="47" t="s">
+      <c r="I5" s="33"/>
+      <c r="J5" s="27" t="s">
         <v>143</v>
       </c>
-      <c r="K5" s="47" t="s">
+      <c r="K5" s="27" t="s">
         <v>144</v>
       </c>
-      <c r="L5" s="42">
+      <c r="L5" s="22">
         <f>'⚙️ 全局核算参数 (Config)'!$C$22</f>
-      </c>
-      <c r="M5" s="43">
-        <f>IF(ISBLANK(I5), '⚙️ 全局核算参数 (Config)'!$B$14, I5)</f>
-      </c>
-      <c r="N5" s="44">
-        <f>ROUND(((D5 * (1 + M5) + L5) / '⚙️ 全局核算参数 (Config)'!$B$6), 2)</f>
-      </c>
-      <c r="O5" s="45">
-        <f>IF(AND(G5&gt;0, F5&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$33 / G5)) * F5, "-")</f>
-      </c>
-      <c r="P5" s="45">
-        <f>IF(AND(G5&gt;0, F5&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$35 / G5)) * F5, "-")</f>
-      </c>
-      <c r="Q5" s="46">
-        <f>IF(M5&lt;'⚙️ 全局核算参数 (Config)'!$B$15, "🚨 穿透红线", IF(M5&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
-      </c>
-    </row>
-    <row r="6" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6" s="35" t="s">
+        <v>0.2</v>
+      </c>
+      <c r="M5" s="23">
+        <f>IF(ISBLANK(I5),'⚙️ 全局核算参数 (Config)'!$B$14,I5)</f>
+        <v>0.15</v>
+      </c>
+      <c r="N5" s="24">
+        <f>ROUND(((D5*(1+M5)+L5)/'⚙️ 全局核算参数 (Config)'!$B$6),2)</f>
+        <v>6.1</v>
+      </c>
+      <c r="O5" s="25">
+        <f>IF(AND(G5&gt;0,F5&gt;0),INT(('⚙️ 全局核算参数 (Config)'!$B$33/G5))*F5,"-")</f>
+        <v>1750</v>
+      </c>
+      <c r="P5" s="25">
+        <f>IF(AND(G5&gt;0,F5&gt;0),INT(('⚙️ 全局核算参数 (Config)'!$B$35/G5))*F5,"-")</f>
+        <v>4250</v>
+      </c>
+      <c r="Q5" s="26" t="str">
+        <f>IF(M5&lt;'⚙️ 全局核算参数 (Config)'!$B$15,"🚨 穿透红线",IF(M5&gt;=0.25,"💎 高毛利款","✅ 利润健康"))</f>
+        <v>✅ 利润健康</v>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1" spans="1:17">
+      <c r="A6" s="15" t="s">
         <v>145</v>
       </c>
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="C6" s="36" t="s">
+      <c r="C6" s="16" t="s">
         <v>147</v>
       </c>
-      <c r="D6" s="37">
+      <c r="D6" s="17">
         <v>24</v>
       </c>
-      <c r="E6" s="38">
+      <c r="E6" s="18">
         <v>300</v>
       </c>
-      <c r="F6" s="38">
+      <c r="F6" s="18">
         <v>20</v>
       </c>
-      <c r="G6" s="39">
+      <c r="G6" s="19">
         <v>0.055</v>
       </c>
-      <c r="H6" s="40">
+      <c r="H6" s="20">
         <v>9.5</v>
       </c>
-      <c r="I6" s="41"/>
-      <c r="J6" s="35" t="s">
+      <c r="I6" s="21"/>
+      <c r="J6" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="K6" s="35" t="s">
+      <c r="K6" s="15" t="s">
         <v>144</v>
       </c>
-      <c r="L6" s="42">
+      <c r="L6" s="22">
         <f>'⚙️ 全局核算参数 (Config)'!$C$22</f>
-      </c>
-      <c r="M6" s="43">
-        <f>IF(ISBLANK(I6), '⚙️ 全局核算参数 (Config)'!$B$14, I6)</f>
-      </c>
-      <c r="N6" s="44">
-        <f>ROUND(((D6 * (1 + M6) + L6) / '⚙️ 全局核算参数 (Config)'!$B$6), 2)</f>
-      </c>
-      <c r="O6" s="45">
-        <f>IF(AND(G6&gt;0, F6&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$33 / G6)) * F6, "-")</f>
-      </c>
-      <c r="P6" s="45">
-        <f>IF(AND(G6&gt;0, F6&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$35 / G6)) * F6, "-")</f>
-      </c>
-      <c r="Q6" s="46">
-        <f>IF(M6&lt;'⚙️ 全局核算参数 (Config)'!$B$15, "🚨 穿透红线", IF(M6&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
-      </c>
-    </row>
-    <row r="7" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A7" s="47" t="s">
+        <v>0.2</v>
+      </c>
+      <c r="M6" s="23">
+        <f>IF(ISBLANK(I6),'⚙️ 全局核算参数 (Config)'!$B$14,I6)</f>
+        <v>0.15</v>
+      </c>
+      <c r="N6" s="24">
+        <f>ROUND(((D6*(1+M6)+L6)/'⚙️ 全局核算参数 (Config)'!$B$6),2)</f>
+        <v>3.86</v>
+      </c>
+      <c r="O6" s="25">
+        <f>IF(AND(G6&gt;0,F6&gt;0),INT(('⚙️ 全局核算参数 (Config)'!$B$33/G6))*F6,"-")</f>
+        <v>10180</v>
+      </c>
+      <c r="P6" s="25">
+        <f>IF(AND(G6&gt;0,F6&gt;0),INT(('⚙️ 全局核算参数 (Config)'!$B$35/G6))*F6,"-")</f>
+        <v>24720</v>
+      </c>
+      <c r="Q6" s="26" t="str">
+        <f>IF(M6&lt;'⚙️ 全局核算参数 (Config)'!$B$15,"🚨 穿透红线",IF(M6&gt;=0.25,"💎 高毛利款","✅ 利润健康"))</f>
+        <v>✅ 利润健康</v>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1" spans="1:17">
+      <c r="A7" s="27" t="s">
         <v>148</v>
       </c>
-      <c r="B7" s="48" t="s">
+      <c r="B7" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="C7" s="48" t="s">
+      <c r="C7" s="28" t="s">
         <v>147</v>
       </c>
-      <c r="D7" s="49">
+      <c r="D7" s="29">
         <v>25</v>
       </c>
-      <c r="E7" s="50">
+      <c r="E7" s="30">
         <v>300</v>
       </c>
-      <c r="F7" s="50">
+      <c r="F7" s="30">
         <v>20</v>
       </c>
-      <c r="G7" s="51">
+      <c r="G7" s="31">
         <v>0.055</v>
       </c>
-      <c r="H7" s="52">
+      <c r="H7" s="32">
         <v>9.5</v>
       </c>
-      <c r="I7" s="53"/>
-      <c r="J7" s="47" t="s">
+      <c r="I7" s="33"/>
+      <c r="J7" s="27" t="s">
         <v>128</v>
       </c>
-      <c r="K7" s="47" t="s">
+      <c r="K7" s="27" t="s">
         <v>144</v>
       </c>
-      <c r="L7" s="42">
+      <c r="L7" s="22">
         <f>'⚙️ 全局核算参数 (Config)'!$C$22</f>
-      </c>
-      <c r="M7" s="43">
-        <f>IF(ISBLANK(I7), '⚙️ 全局核算参数 (Config)'!$B$14, I7)</f>
-      </c>
-      <c r="N7" s="44">
-        <f>ROUND(((D7 * (1 + M7) + L7) / '⚙️ 全局核算参数 (Config)'!$B$6), 2)</f>
-      </c>
-      <c r="O7" s="45">
-        <f>IF(AND(G7&gt;0, F7&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$33 / G7)) * F7, "-")</f>
-      </c>
-      <c r="P7" s="45">
-        <f>IF(AND(G7&gt;0, F7&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$35 / G7)) * F7, "-")</f>
-      </c>
-      <c r="Q7" s="46">
-        <f>IF(M7&lt;'⚙️ 全局核算参数 (Config)'!$B$15, "🚨 穿透红线", IF(M7&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
+        <v>0.2</v>
+      </c>
+      <c r="M7" s="23">
+        <f>IF(ISBLANK(I7),'⚙️ 全局核算参数 (Config)'!$B$14,I7)</f>
+        <v>0.15</v>
+      </c>
+      <c r="N7" s="24">
+        <f>ROUND(((D7*(1+M7)+L7)/'⚙️ 全局核算参数 (Config)'!$B$6),2)</f>
+        <v>4.02</v>
+      </c>
+      <c r="O7" s="25">
+        <f>IF(AND(G7&gt;0,F7&gt;0),INT(('⚙️ 全局核算参数 (Config)'!$B$33/G7))*F7,"-")</f>
+        <v>10180</v>
+      </c>
+      <c r="P7" s="25">
+        <f>IF(AND(G7&gt;0,F7&gt;0),INT(('⚙️ 全局核算参数 (Config)'!$B$35/G7))*F7,"-")</f>
+        <v>24720</v>
+      </c>
+      <c r="Q7" s="26" t="str">
+        <f>IF(M7&lt;'⚙️ 全局核算参数 (Config)'!$B$15,"🚨 穿透红线",IF(M7&gt;=0.25,"💎 高毛利款","✅ 利润健康"))</f>
+        <v>✅ 利润健康</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:I9"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -2203,235 +2919,283 @@
     <col min="7" max="9" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="54" t="s">
+    <row r="1" ht="36" customHeight="1" spans="1:9">
+      <c r="A1" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
-    </row>
-    <row r="2" ht="24" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="55" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+    </row>
+    <row r="2" ht="24" customHeight="1" spans="1:9">
+      <c r="A2" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="56" t="s">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="56"/>
-    </row>
-    <row r="3" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="57" t="s">
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+    </row>
+    <row r="3" ht="26" customHeight="1" spans="1:9">
+      <c r="A3" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="B3" s="57" t="s">
+      <c r="B3" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="C3" s="57" t="s">
+      <c r="C3" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="D3" s="57" t="s">
+      <c r="D3" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="E3" s="57" t="s">
+      <c r="E3" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="F3" s="57" t="s">
+      <c r="F3" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="G3" s="57" t="s">
+      <c r="G3" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="H3" s="57" t="s">
+      <c r="H3" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="I3" s="57" t="s">
+      <c r="I3" s="4" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="58">
+    <row r="4" ht="22" customHeight="1" spans="1:9">
+      <c r="A4" s="5">
         <v>1</v>
       </c>
-      <c r="B4" s="58">
+      <c r="B4" s="5" t="str">
         <f>'📦 商品出厂底价库 (Products)'!A2</f>
-      </c>
-      <c r="C4" s="59">
+        <v>ST-2026-A</v>
+      </c>
+      <c r="C4" s="6" t="str">
         <f>'📦 商品出厂底价库 (Products)'!C2</f>
-      </c>
-      <c r="D4" s="60">
+        <v>Aluminum Alloy Precision Bracket (铝合金精密五金支架)</v>
+      </c>
+      <c r="D4" s="7">
         <f>'📦 商品出厂底价库 (Products)'!E2</f>
-      </c>
-      <c r="E4" s="61">
+        <v>600</v>
+      </c>
+      <c r="E4" s="8">
         <f>'📦 商品出厂底价库 (Products)'!N2</f>
-      </c>
-      <c r="F4" s="60">
+        <v>2.5</v>
+      </c>
+      <c r="F4" s="7">
         <f>'📦 商品出厂底价库 (Products)'!F2</f>
-      </c>
-      <c r="G4" s="60">
+        <v>50</v>
+      </c>
+      <c r="G4" s="7">
         <f>'📦 商品出厂底价库 (Products)'!O2</f>
-      </c>
-      <c r="H4" s="60">
+        <v>31100</v>
+      </c>
+      <c r="H4" s="7">
         <f>'📦 商品出厂底价库 (Products)'!P2</f>
-      </c>
-      <c r="I4" s="58">
+        <v>75550</v>
+      </c>
+      <c r="I4" s="5" t="str">
         <f>'📦 商品出厂底价库 (Products)'!J2</f>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="62">
+        <v>20-25 Days</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:9">
+      <c r="A5" s="9">
         <v>2</v>
       </c>
-      <c r="B5" s="62">
+      <c r="B5" s="9" t="str">
         <f>'📦 商品出厂底价库 (Products)'!A3</f>
-      </c>
-      <c r="C5" s="63">
+        <v>ST-2026-B</v>
+      </c>
+      <c r="C5" s="10" t="str">
         <f>'📦 商品出厂底价库 (Products)'!C3</f>
-      </c>
-      <c r="D5" s="64">
+        <v>Stainless Steel Hex Fastener Screws (不锈钢沉头紧固件螺丝)</v>
+      </c>
+      <c r="D5" s="11">
         <f>'📦 商品出厂底价库 (Products)'!E3</f>
-      </c>
-      <c r="E5" s="65">
+        <v>5000</v>
+      </c>
+      <c r="E5" s="12">
         <f>'📦 商品出厂底价库 (Products)'!N3</f>
-      </c>
-      <c r="F5" s="64">
+        <v>0.17</v>
+      </c>
+      <c r="F5" s="11">
         <f>'📦 商品出厂底价库 (Products)'!F3</f>
-      </c>
-      <c r="G5" s="64">
+        <v>1000</v>
+      </c>
+      <c r="G5" s="11">
         <f>'📦 商品出厂底价库 (Products)'!O3</f>
-      </c>
-      <c r="H5" s="64">
+        <v>1400000</v>
+      </c>
+      <c r="H5" s="11">
         <f>'📦 商品出厂底价库 (Products)'!P3</f>
-      </c>
-      <c r="I5" s="62">
+        <v>3400000</v>
+      </c>
+      <c r="I5" s="9" t="str">
         <f>'📦 商品出厂底价库 (Products)'!J3</f>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="58">
+        <v>15-20 Days</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="1:9">
+      <c r="A6" s="5">
         <v>3</v>
       </c>
-      <c r="B6" s="58">
+      <c r="B6" s="5" t="str">
         <f>'📦 商品出厂底价库 (Products)'!A4</f>
-      </c>
-      <c r="C6" s="59">
+        <v>ERG-PRO-V2</v>
+      </c>
+      <c r="C6" s="6" t="str">
         <f>'📦 商品出厂底价库 (Products)'!C4</f>
-      </c>
-      <c r="D6" s="60">
+        <v>Ergonomic Mesh Office Chair (高档网布人体工学办公椅)</v>
+      </c>
+      <c r="D6" s="7">
         <f>'📦 商品出厂底价库 (Products)'!E4</f>
-      </c>
-      <c r="E6" s="61">
+        <v>50</v>
+      </c>
+      <c r="E6" s="8">
         <f>'📦 商品出厂底价库 (Products)'!N4</f>
-      </c>
-      <c r="F6" s="60">
+        <v>32.15</v>
+      </c>
+      <c r="F6" s="7">
         <f>'📦 商品出厂底价库 (Products)'!F4</f>
-      </c>
-      <c r="G6" s="60">
+        <v>1</v>
+      </c>
+      <c r="G6" s="7">
         <f>'📦 商品出厂底价库 (Products)'!O4</f>
-      </c>
-      <c r="H6" s="60">
+        <v>175</v>
+      </c>
+      <c r="H6" s="7">
         <f>'📦 商品出厂底价库 (Products)'!P4</f>
-      </c>
-      <c r="I6" s="58">
+        <v>425</v>
+      </c>
+      <c r="I6" s="5" t="str">
         <f>'📦 商品出厂底价库 (Products)'!J4</f>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="62">
+        <v>30-35 Days</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1" spans="1:9">
+      <c r="A7" s="9">
         <v>4</v>
       </c>
-      <c r="B7" s="62">
+      <c r="B7" s="9" t="str">
         <f>'📦 商品出厂底价库 (Products)'!A5</f>
-      </c>
-      <c r="C7" s="63">
+        <v>AL-BASE-99</v>
+      </c>
+      <c r="C7" s="10" t="str">
         <f>'📦 商品出厂底价库 (Products)'!C5</f>
-      </c>
-      <c r="D7" s="64">
+        <v>Die-casting Aluminum 5-Star Base (高压铸铝合金五星椅脚)</v>
+      </c>
+      <c r="D7" s="11">
         <f>'📦 商品出厂底价库 (Products)'!E5</f>
-      </c>
-      <c r="E7" s="65">
+        <v>200</v>
+      </c>
+      <c r="E7" s="12">
         <f>'📦 商品出厂底价库 (Products)'!N5</f>
-      </c>
-      <c r="F7" s="64">
+        <v>6.1</v>
+      </c>
+      <c r="F7" s="11">
         <f>'📦 商品出厂底价库 (Products)'!F5</f>
-      </c>
-      <c r="G7" s="64">
+        <v>5</v>
+      </c>
+      <c r="G7" s="11">
         <f>'📦 商品出厂底价库 (Products)'!O5</f>
-      </c>
-      <c r="H7" s="64">
+        <v>1750</v>
+      </c>
+      <c r="H7" s="11">
         <f>'📦 商品出厂底价库 (Products)'!P5</f>
-      </c>
-      <c r="I7" s="62">
+        <v>4250</v>
+      </c>
+      <c r="I7" s="9" t="str">
         <f>'📦 商品出厂底价库 (Products)'!J5</f>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="58">
+        <v>25-30 Days</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1" spans="1:9">
+      <c r="A8" s="5">
         <v>5</v>
       </c>
-      <c r="B8" s="58">
+      <c r="B8" s="5" t="str">
         <f>'📦 商品出厂底价库 (Products)'!A6</f>
-      </c>
-      <c r="C8" s="59">
+        <v>HD-ARM-08</v>
+      </c>
+      <c r="C8" s="6" t="str">
         <f>'📦 商品出厂底价库 (Products)'!C6</f>
-      </c>
-      <c r="D8" s="60">
+        <v>3D Adjustable PU Armrest Set (3D多功能升降PU扶手套装)</v>
+      </c>
+      <c r="D8" s="7">
         <f>'📦 商品出厂底价库 (Products)'!E6</f>
-      </c>
-      <c r="E8" s="61">
+        <v>300</v>
+      </c>
+      <c r="E8" s="8">
         <f>'📦 商品出厂底价库 (Products)'!N6</f>
-      </c>
-      <c r="F8" s="60">
+        <v>3.86</v>
+      </c>
+      <c r="F8" s="7">
         <f>'📦 商品出厂底价库 (Products)'!F6</f>
-      </c>
-      <c r="G8" s="60">
+        <v>20</v>
+      </c>
+      <c r="G8" s="7">
         <f>'📦 商品出厂底价库 (Products)'!O6</f>
-      </c>
-      <c r="H8" s="60">
+        <v>10180</v>
+      </c>
+      <c r="H8" s="7">
         <f>'📦 商品出厂底价库 (Products)'!P6</f>
-      </c>
-      <c r="I8" s="58">
+        <v>24720</v>
+      </c>
+      <c r="I8" s="5" t="str">
         <f>'📦 商品出厂底价库 (Products)'!J6</f>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="62">
+        <v>20-25 Days</v>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1" spans="1:9">
+      <c r="A9" s="9">
         <v>6</v>
       </c>
-      <c r="B9" s="62">
+      <c r="B9" s="9" t="str">
         <f>'📦 商品出厂底价库 (Products)'!A7</f>
-      </c>
-      <c r="C9" s="63">
+        <v>HD-ARM-09</v>
+      </c>
+      <c r="C9" s="10" t="str">
         <f>'📦 商品出厂底价库 (Products)'!C7</f>
-      </c>
-      <c r="D9" s="64">
+        <v>3D Adjustable PU Armrest Set (3D多功能升降PU扶手套装)</v>
+      </c>
+      <c r="D9" s="11">
         <f>'📦 商品出厂底价库 (Products)'!E7</f>
-      </c>
-      <c r="E9" s="65">
+        <v>300</v>
+      </c>
+      <c r="E9" s="12">
         <f>'📦 商品出厂底价库 (Products)'!N7</f>
-      </c>
-      <c r="F9" s="64">
+        <v>4.02</v>
+      </c>
+      <c r="F9" s="11">
         <f>'📦 商品出厂底价库 (Products)'!F7</f>
-      </c>
-      <c r="G9" s="64">
+        <v>20</v>
+      </c>
+      <c r="G9" s="11">
         <f>'📦 商品出厂底价库 (Products)'!O7</f>
-      </c>
-      <c r="H9" s="64">
+        <v>10180</v>
+      </c>
+      <c r="H9" s="11">
         <f>'📦 商品出厂底价库 (Products)'!P7</f>
-      </c>
-      <c r="I9" s="62">
+        <v>24720</v>
+      </c>
+      <c r="I9" s="9" t="str">
         <f>'📦 商品出厂底价库 (Products)'!J7</f>
+        <v>20-25 Days</v>
       </c>
     </row>
   </sheetData>
@@ -2441,6 +3205,7 @@
     <mergeCell ref="F2:I2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>